<commit_message>
Apply three game design videos to Politics
Adds the lessons document (form follows function, core mechanic,
gameplay loops, signs and feedback, difficulty flow, feature creep,
tutorial, screen readability) and a signs-and-feedback sheet in the
asset tracker listing the sounds and animations each action needs.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013ScbAjnnHvWadm23zH5KKB
</commit_message>
<xml_diff>
--- a/politics-assets/Politics_assets.xlsx
+++ b/politics-assets/Politics_assets.xlsx
@@ -8,15 +8,17 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inventaire" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sons à sourcer" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Textes à écrire" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide GSG" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Signes et feedback" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sons à sourcer" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Textes à écrire" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide GSG" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventaire'!$A$1:$J$18</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Sons à sourcer'!$A$1:$I$10</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Textes à écrire'!$A$1:$F$6</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Guide GSG'!$A$1:$E$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventaire'!$A$1:$K$18</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Signes et feedback'!$A$1:$J$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Sons à sourcer'!$A$1:$I$17</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Textes à écrire'!$A$1:$F$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Guide GSG'!$A$1:$E$13</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -63,13 +65,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -436,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J18"/>
+  <dimension ref="A1:K18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -449,6 +454,7 @@
     <col width="20" customWidth="1" min="8" max="8"/>
     <col width="20" customWidth="1" min="9" max="9"/>
     <col width="30" customWidth="1" min="10" max="10"/>
+    <col width="40" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -502,6 +508,11 @@
           <t>Notes</t>
         </is>
       </c>
+      <c r="K1" s="3" t="inlineStr">
+        <is>
+          <t>Fonction (ce que l'asset dit au joueur)</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -554,6 +565,11 @@
           <t>Confirmer le chemin exact</t>
         </is>
       </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>Journaliste exigeant mais juste (mordant 6)</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -602,6 +618,11 @@
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr"/>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>Radio libre, proche des quartiers populaires (mordant 4)</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -650,6 +671,11 @@
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr"/>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>Le plus dur, la télévision (mordant 7)</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -698,6 +724,11 @@
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr"/>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>Hebdo rural bienveillant (mordant 3)</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -1238,6 +1269,11 @@
           <t>Voir onglet Sons à sourcer</t>
         </is>
       </c>
+      <c r="K16" s="2" t="inlineStr">
+        <is>
+          <t>La salle vous suit</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -1290,6 +1326,11 @@
           <t>Pas encore de CC0 sûr</t>
         </is>
       </c>
+      <c r="K17" s="2" t="inlineStr">
+        <is>
+          <t>La salle vous rejette</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -1340,7 +1381,7 @@
       <c r="J18" s="2" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J18"/>
+  <autoFilter ref="A1:K18"/>
   <dataValidations count="1">
     <dataValidation sqref="H2:H500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Manquant,Recherche,Candidat trouvé,Livré à la session Godot,Intégré,Final,Provisoire"</formula1>
@@ -1356,7 +1397,871 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I10"/>
+  <dimension ref="A1:J16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="11" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="32" customWidth="1" min="4" max="4"/>
+    <col width="36" customWidth="1" min="5" max="5"/>
+    <col width="36" customWidth="1" min="6" max="6"/>
+    <col width="34" customWidth="1" min="7" max="7"/>
+    <col width="30" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Moment</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Action du joueur</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Signe avant l'action</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Feedback si réussite</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Feedback si échec</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Son(s) nécessaire(s)</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Visuel / animation nécessaire</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Existe déjà ?</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Statut</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>SF-01</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Mandat</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Proposer une mesure</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Coût, délai et élus concernés affichés</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Dossier qui s'ouvre, son de papier</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Message clair : pourquoi c'est impossible</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>Feuilles de papier</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>Dossier qui s'ouvre</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>à confirmer</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>Manquant</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>SF-02</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Mandat</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Inscrire à l'ordre du jour</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Date de la prochaine séance</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Tampon « Inscrit »</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>Tampon encreur</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>Tampon animé</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>à confirmer</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>Manquant</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>SF-03</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Mandat</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Rencontrer un élu</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Relation et ambition visibles sur la carte</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Expression qui s'adoucit, chiffre vert</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Expression fermée, chiffre rouge</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>Discussion feutrée, porte de bureau</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>Expressions (existent)</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>En partie</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>À compléter</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>SF-04</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Mandat</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Faire voter en conseil</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Décompte prévu : pour, contre, incertains</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>Coup de marteau, applaudissements de la majorité, tampon « Adoptée »</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>Brouhaha, tampon « Rejetée », liste des élus qui ont lâché</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>Marteau de séance, applaudissements polis, brouhaha de conseil</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>Tampon Adoptée / Rejetée, légère secousse</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>à confirmer</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>Manquant</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>SF-05</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Mandat</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Nommer un adjoint</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Compétence de l'élu face à la délégation</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Écharpe qui apparaît, bonus affiché</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>Malus affiché si incompétent</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>Petit carillon</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>Médaillon de délégation</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>En partie</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>À compléter</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>SF-06</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Mandat</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Répondre à une doléance</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Lettre en attente, ancienneté visible</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>Lettre cachetée envoyée, quartier qui verdit</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>Lettre qui jaunit, alerte au bout de 2 mois</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>Enveloppe, cachet de cire</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>Lettre qui jaunit</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>à confirmer</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>Manquant</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>SF-07</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Mandat</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Voter le budget / les impôts</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Effet prévu par quartier (infobulle)</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>Calculatrice, chiffres qui se figent</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>Grogne affichée sur la carte</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>Machine à calculer à rouleau</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>Carte qui rougit par quartier</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>à confirmer</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>Manquant</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>SF-08</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Mandat</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Passer au mois suivant</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>Bouton « mois suivant », alertes non lues</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>Rotative, journal qui tombe</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>Rotative d'imprimerie</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>Journal qui tombe sur le bureau</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>En partie (journal)</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>À compléter</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>SF-09</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Mandat</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>(subi) Un élu quitte la majorité</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>« Bruits de couloir » un mois avant</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>Porte qui claque, portrait qui change de couleur</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>Porte qui claque</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>Portrait qui bascule</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>Manquant</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>SF-10</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Mandat</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>(subi) Cortège, manifestation</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>Tension du quartier affichée</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>Cortège qui se disperse si on négocie</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>Slogans, sifflets</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>Foule qui scande, sifflets</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>Cortège sur la carte (existe)</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>En partie</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>À compléter</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>SF-11</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Campagne</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Répondre à un journaliste</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Chance, gain, risque (existent)</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>Hochement de tête, stylo qui note, chiffre vert</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>Sourcil levé, relance, chiffre rouge</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>Stylo sur papier, machine à écrire (presse écrite), jingle radio, générique TV</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>Expressions (existent)</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>En partie</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>À compléter</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>SF-12</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Campagne</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Meeting de quartier</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>Souci du quartier affiché</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>Applaudissements qui montent</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>Huées, chaises qui grincent</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>Applaudissements, huées, chaises</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>Salle (existe)</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>En partie</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>Candidat trouvé</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>SF-13</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Campagne</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Débat face à Carminati</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>Le pire de votre bilan est annoncé</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>Cadrage qui se resserre sur vous, public qui réagit</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>Cadrage sur Carminati, rires du public</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>Générique de débat, réactions du public</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>Cadrages (à faire)</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>En partie</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>À compléter</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>SF-14</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Campagne</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>Tracts, sondages</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>Coût et quartier ciblé</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>Ronéo, sondage qui monte</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>Sondage qui baisse</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>Ronéotypeuse</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>Courbe animée</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>à confirmer</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="inlineStr">
+        <is>
+          <t>Manquant</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>SF-15</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Élection</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Soirée électorale (13 mars 1983)</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>Compte à rebours de 20 h</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>Foule en liesse, une de journal « Réélu »</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>Silence, une « Battu »</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>Foule en liesse, générique de soirée électorale TV</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>Résultats quartier par quartier, une de journal</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>à confirmer</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t>Manquant</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:J16"/>
+  <dataValidations count="1">
+    <dataValidation sqref="J2:J500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Manquant,À compléter,Candidat trouvé,Livré à la session Godot,Intégré,Final"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -1832,8 +2737,281 @@
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>SND-020</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Marteau de séance (vote)</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>À chercher</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr"/>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>CC0 visé</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr"/>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>Recherche</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>SF-04</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>SND-021</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Tampon encreur (Adoptée, Inscrit)</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>À chercher</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr"/>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>CC0 visé</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr"/>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>Recherche</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>SF-02, SF-04</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>SND-022</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Rotative d'imprimerie (journal du mois)</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>À chercher</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr"/>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>CC0 visé</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr"/>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>Recherche</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>SF-08</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>SND-023</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Porte qui claque (défection)</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>À chercher</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr"/>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>CC0 visé</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr"/>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>Recherche</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>SF-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>SND-024</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Brouhaha de conseil municipal</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>À chercher</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr"/>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>CC0 visé</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr"/>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>Recherche</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>SF-04</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>SND-025</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Chaises qui grincent, salle des fêtes</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>À chercher</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr"/>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>CC0 visé</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr"/>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>Recherche</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>SF-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>SND-026</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Machine à calculer à rouleau / ronéotypeuse</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>À chercher</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr"/>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>CC0 visé</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr"/>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>Recherche</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>SF-07, SF-14</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I10"/>
+  <autoFilter ref="A1:I17"/>
   <dataValidations count="1">
     <dataValidation sqref="H2:H500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Manquant,Recherche,Candidat trouvé,Livré à la session Godot,Intégré,Final,Provisoire"</formula1>
@@ -1843,7 +3021,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2059,7 +3237,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Add lessons from the Racine management game video
Game pillars proposal, single UI reference (Crusader Kings 3), visible
commune mood through the town square and mayor's office, music brief
with a municipal brass band signature, and new tracker rows.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013ScbAjnnHvWadm23zH5KKB
</commit_message>
<xml_diff>
--- a/politics-assets/Politics_assets.xlsx
+++ b/politics-assets/Politics_assets.xlsx
@@ -14,7 +14,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide GSG" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventaire'!$A$1:$K$18</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventaire'!$A$1:$K$24</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Signes et feedback'!$A$1:$J$16</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Sons à sourcer'!$A$1:$I$17</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Textes à écrire'!$A$1:$F$6</definedName>
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K18"/>
+  <dimension ref="A1:K24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -777,6 +777,7 @@
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr"/>
+      <c r="K6" s="2" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -829,6 +830,7 @@
           <t>Chemin déduit</t>
         </is>
       </c>
+      <c r="K7" s="2" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -881,6 +883,7 @@
           <t>Chemin déduit</t>
         </is>
       </c>
+      <c r="K8" s="2" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -929,6 +932,7 @@
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr"/>
+      <c r="K9" s="2" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -977,6 +981,7 @@
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr"/>
+      <c r="K10" s="2" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1025,6 +1030,7 @@
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr"/>
+      <c r="K11" s="2" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1073,6 +1079,7 @@
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr"/>
+      <c r="K12" s="2" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -1121,6 +1128,7 @@
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr"/>
+      <c r="K13" s="2" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -1169,6 +1177,7 @@
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr"/>
+      <c r="K14" s="2" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -1217,6 +1226,7 @@
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr"/>
+      <c r="K15" s="2" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -1379,9 +1389,340 @@
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr"/>
+      <c r="K18" s="2" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>IMG-020</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>Décor</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>Place de la mairie, 4 états d'opinion (fête, normal, tendu, grève)</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>à définir</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>webp</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>Higgsfield</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>Abonnement Higgsfield</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>Manquant</t>
+        </is>
+      </c>
+      <c r="I19" s="2" t="inlineStr">
+        <is>
+          <t>Session cloud (brief) + Godot (intégration)</t>
+        </is>
+      </c>
+      <c r="J19" s="2" t="inlineStr">
+        <is>
+          <t>Narrative design, voir Lecons § 10.3</t>
+        </is>
+      </c>
+      <c r="K19" s="2" t="inlineStr">
+        <is>
+          <t>L'opinion de la commune se voit sans chiffre</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>IMG-021</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>Décor</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>Bureau du maire qui se remplit au fil du mandat (dossiers, coupures encadrées, lettres en souffrance)</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>à définir</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>webp</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>Higgsfield</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>Abonnement Higgsfield</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>Manquant</t>
+        </is>
+      </c>
+      <c r="I20" s="2" t="inlineStr">
+        <is>
+          <t>Session cloud (brief)</t>
+        </is>
+      </c>
+      <c r="J20" s="2" t="inlineStr">
+        <is>
+          <t>§ 10.3</t>
+        </is>
+      </c>
+      <c r="K20" s="2" t="inlineStr">
+        <is>
+          <t>Le bilan du mandat se voit</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>IMG-022</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>Icônes</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>Icônes des ressources et des modes de carte, style CK3</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>à définir</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>png/svg</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>à définir</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>à définir</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>Manquant</t>
+        </is>
+      </c>
+      <c r="I21" s="2" t="inlineStr">
+        <is>
+          <t>Session cloud (recherche)</t>
+        </is>
+      </c>
+      <c r="J21" s="2" t="inlineStr">
+        <is>
+          <t>§ 10.5</t>
+        </is>
+      </c>
+      <c r="K21" s="2" t="inlineStr">
+        <is>
+          <t>Lire une ressource d'un coup d'œil</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>MUS-001</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>Musique</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>Thèmes mairie et campagne avec cuivres de fanfare municipale en signature</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>à confirmer</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>ogg</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>à définir</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>à définir</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>Recherche</t>
+        </is>
+      </c>
+      <c r="I22" s="2" t="inlineStr">
+        <is>
+          <t>Session cloud</t>
+        </is>
+      </c>
+      <c r="J22" s="2" t="inlineStr">
+        <is>
+          <t>Brief § 10.5 ; vérifier ce qui existe déjà</t>
+        </is>
+      </c>
+      <c r="K22" s="2" t="inlineStr">
+        <is>
+          <t>L'ambiance du mandat (fête ou grève)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>DOC-001</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>Document</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>Bible graphique de Politics</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>politics-assets/</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>md</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>Session cloud + Godot</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>Projet</t>
+        </is>
+      </c>
+      <c r="H23" s="2" t="inlineStr">
+        <is>
+          <t>Manquant</t>
+        </is>
+      </c>
+      <c r="I23" s="2" t="inlineStr">
+        <is>
+          <t>Session cloud (brouillon)</t>
+        </is>
+      </c>
+      <c r="J23" s="2" t="inlineStr">
+        <is>
+          <t>Besoin de captures du jeu</t>
+        </is>
+      </c>
+      <c r="K23" s="2" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>DOC-002</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>Document</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>Game pillars de Politics</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>Lecons_videos_game_design.md § 10.1</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>md</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>Session cloud</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>Projet</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>Provisoire</t>
+        </is>
+      </c>
+      <c r="I24" s="2" t="inlineStr">
+        <is>
+          <t>Yannick (validation)</t>
+        </is>
+      </c>
+      <c r="J24" s="2" t="inlineStr"/>
+      <c r="K24" s="2" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K18"/>
+  <autoFilter ref="A1:K24"/>
   <dataValidations count="1">
     <dataValidation sqref="H2:H500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Manquant,Recherche,Candidat trouvé,Livré à la session Godot,Intégré,Final,Provisoire"</formula1>
@@ -3027,7 +3368,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -3223,6 +3564,38 @@
       <c r="F6" s="2" t="inlineStr">
         <is>
           <t>Pilier 4 du guide GSG</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>TXT-105</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>à définir (événements)</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Brouilles entre élus : deux adjoints qui se fâchent, réconciliation possible</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>8 à 10 événements</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Manquant</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Lecons § 10.4</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add lessons from the 12 game design lessons video
USP and pitch proposal, singularity questions for the author, enemies
as the source of fun (Carminati present through the whole term), save
design, scope and demo, and a precise playtest protocol.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013ScbAjnnHvWadm23zH5KKB
</commit_message>
<xml_diff>
--- a/politics-assets/Politics_assets.xlsx
+++ b/politics-assets/Politics_assets.xlsx
@@ -14,10 +14,10 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide GSG" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventaire'!$A$1:$K$24</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventaire'!$A$1:$K$27</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Signes et feedback'!$A$1:$J$16</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Sons à sourcer'!$A$1:$I$17</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Textes à écrire'!$A$1:$F$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Textes à écrire'!$A$1:$F$8</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Guide GSG'!$A$1:$E$13</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K24"/>
+  <dimension ref="A1:K27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -1721,8 +1721,171 @@
       <c r="J24" s="2" t="inlineStr"/>
       <c r="K24" s="2" t="inlineStr"/>
     </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>DOC-003</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>Document</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>Pitch du jeu (long et court)</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>Lecons_videos_game_design.md § 11.3</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>md</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>Session cloud</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>Projet</t>
+        </is>
+      </c>
+      <c r="H25" s="2" t="inlineStr">
+        <is>
+          <t>Provisoire</t>
+        </is>
+      </c>
+      <c r="I25" s="2" t="inlineStr">
+        <is>
+          <t>Yannick (validation)</t>
+        </is>
+      </c>
+      <c r="J25" s="2" t="inlineStr"/>
+      <c r="K25" s="2" t="inlineStr">
+        <is>
+          <t>Donner envie en une minute</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>DOC-004</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>Document</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>Protocole et questionnaire de playtest</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>à rédiger</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>md</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>Session cloud</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>Projet</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>Manquant</t>
+        </is>
+      </c>
+      <c r="I26" s="2" t="inlineStr">
+        <is>
+          <t>Session cloud</t>
+        </is>
+      </c>
+      <c r="J26" s="2" t="inlineStr">
+        <is>
+          <t>§ 11.8</t>
+        </is>
+      </c>
+      <c r="K26" s="2" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>DOC-005</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>Maquettes</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>Maquettes d'écrans avant code (fiche de quartier, trois horizons, front électoral)</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>à faire</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>png</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>Session cloud</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t>Projet</t>
+        </is>
+      </c>
+      <c r="H27" s="2" t="inlineStr">
+        <is>
+          <t>Manquant</t>
+        </is>
+      </c>
+      <c r="I27" s="2" t="inlineStr">
+        <is>
+          <t>Session cloud</t>
+        </is>
+      </c>
+      <c r="J27" s="2" t="inlineStr">
+        <is>
+          <t>§ 11.4, à valider par Yannick avant code</t>
+        </is>
+      </c>
+      <c r="K27" s="2" t="inlineStr">
+        <is>
+          <t>Juger une idée avant de la coder</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K24"/>
+  <autoFilter ref="A1:K27"/>
   <dataValidations count="1">
     <dataValidation sqref="H2:H500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Manquant,Recherche,Candidat trouvé,Livré à la session Godot,Intégré,Final,Provisoire"</formula1>
@@ -3368,7 +3531,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:F8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -3568,39 +3731,71 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="2" t="inlineStr">
         <is>
           <t>TXT-105</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B7" s="2" t="inlineStr">
         <is>
           <t>à définir (événements)</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C7" s="2" t="inlineStr">
         <is>
           <t>Brouilles entre élus : deux adjoints qui se fâchent, réconciliation possible</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="D7" s="2" t="inlineStr">
         <is>
           <t>8 à 10 événements</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="E7" s="2" t="inlineStr">
         <is>
           <t>Manquant</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
+      <c r="F7" s="2" t="inlineStr">
         <is>
           <t>Lecons § 10.4</t>
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>TXT-106</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>à définir (presse, conseil)</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Carminati présent pendant tout le mandat : déclarations dans la presse, interventions au conseil</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>1 à 2 par trimestre</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>Manquant</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>Lecons § 11.5</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F6"/>
+  <autoFilter ref="A1:F8"/>
   <dataValidations count="1">
     <dataValidation sqref="E2:E500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Manquant,Recherche,Candidat trouvé,Livré à la session Godot,Intégré,Final,Provisoire"</formula1>

</xml_diff>

<commit_message>
Align Politics docs and tracker with the real game inventory
Corrects the framing (play starts 1 January 1980 in Saint-Aubin-sur-Viere),
replaces the guessed inventory with the one sent by the Godot session,
adds the priority sounds sheet and fills the feedback sheet's existing
state column.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013ScbAjnnHvWadm23zH5KKB
</commit_message>
<xml_diff>
--- a/politics-assets/Politics_assets.xlsx
+++ b/politics-assets/Politics_assets.xlsx
@@ -9,16 +9,18 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inventaire" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Signes et feedback" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sons à sourcer" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Textes à écrire" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide GSG" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sons prioritaires" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sons à sourcer" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Textes à écrire" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide GSG" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventaire'!$A$1:$K$27</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventaire'!$A$1:$L$38</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Signes et feedback'!$A$1:$J$16</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Sons à sourcer'!$A$1:$I$17</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Textes à écrire'!$A$1:$F$8</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Guide GSG'!$A$1:$E$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Sons prioritaires'!$A$1:$G$35</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Sons à sourcer'!$A$1:$I$17</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Textes à écrire'!$A$1:$F$8</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Guide GSG'!$A$1:$E$13</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -65,7 +67,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -76,6 +78,7 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -441,20 +444,21 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K27"/>
+  <dimension ref="A1:L38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
-    <col width="11" customWidth="1" min="2" max="2"/>
-    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="48" customWidth="1" min="3" max="3"/>
     <col width="34" customWidth="1" min="4" max="4"/>
-    <col width="7" customWidth="1" min="5" max="5"/>
-    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
     <col width="18" customWidth="1" min="7" max="7"/>
-    <col width="20" customWidth="1" min="8" max="8"/>
-    <col width="20" customWidth="1" min="9" max="9"/>
-    <col width="30" customWidth="1" min="10" max="10"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="9" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
     <col width="40" customWidth="1" min="11" max="11"/>
+    <col width="34" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -500,15 +504,20 @@
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
+          <t>Priorité</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
           <t>Responsable</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
-      <c r="K1" s="3" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Fonction (ce que l'asset dit au joueur)</t>
         </is>
@@ -527,49 +536,42 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Odile Ferrand (La Dépêche), 4 expressions</t>
+          <t>11 personnages, 12 expressions (Vasseur, Delorme, Giscard, adjoint_travaux, contestataire, Carminati, opposition_moderee, conseiller_rural, secretaire_general, prefet, president_cg)</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>à confirmer</t>
+          <t>game/ui/portraits/&lt;id&gt;/&lt;expression&gt;.png</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>webp</t>
+          <t>PNG 256×256 RGBA détouré</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Higgsfield</t>
+          <t>3 planches fournies par Yannick, 8 par Higgsfield</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Abonnement Higgsfield</t>
+          <t>Projet / Higgsfield</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>Intégré</t>
-        </is>
-      </c>
-      <c r="I2" s="2" t="inlineStr">
-        <is>
-          <t>Session Godot</t>
-        </is>
-      </c>
+          <t>Final</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr"/>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>Confirmer le chemin exact</t>
-        </is>
-      </c>
-      <c r="K2" s="2" t="inlineStr">
-        <is>
-          <t>Journaliste exigeant mais juste (mordant 6)</t>
-        </is>
-      </c>
+          <t>Godot</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr"/>
+      <c r="L2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -584,17 +586,17 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Thierry Vannier (Radio Vière FM), 4 expressions</t>
+          <t>4 journalistes × 4 expressions (neutre, sourire, incrédule, agacé)</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>à confirmer</t>
+          <t>game/ui/portraits/journaliste_*/</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>webp</t>
+          <t>PNG 256×256</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
@@ -604,23 +606,24 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Abonnement Higgsfield</t>
+          <t>Higgsfield</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>Intégré</t>
-        </is>
-      </c>
-      <c r="I3" s="2" t="inlineStr">
-        <is>
-          <t>Session Godot</t>
-        </is>
-      </c>
-      <c r="J3" s="2" t="inlineStr"/>
-      <c r="K3" s="2" t="inlineStr">
-        <is>
-          <t>Radio libre, proche des quartiers populaires (mordant 4)</t>
+          <t>Final</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr"/>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>Godot</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr"/>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>Le mordant de chaque média</t>
         </is>
       </c>
     </row>
@@ -637,17 +640,17 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Michel Garnier (FR3 Région), 4 expressions</t>
+          <t>5 porte-parole de quartier (citoyen_&lt;quartier&gt;), neutre seulement</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>à confirmer</t>
+          <t>game/ui/portraits/citoyen_*/</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>webp</t>
+          <t>PNG 256×256</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
@@ -657,23 +660,32 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Abonnement Higgsfield</t>
+          <t>Higgsfield</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>Intégré</t>
+          <t>Provisoire</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>Session Godot</t>
-        </is>
-      </c>
-      <c r="J4" s="2" t="inlineStr"/>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>Cloud (brief) / Godot</t>
+        </is>
+      </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>Le plus dur, la télévision (mordant 7)</t>
+          <t>Il faut 4 expressions : ils interpellent en meeting</t>
+        </is>
+      </c>
+      <c r="L4" s="2" t="inlineStr">
+        <is>
+          <t>La salle vous suit ou non</t>
         </is>
       </c>
     </row>
@@ -690,45 +702,50 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Lucien Brac (L'Écho du canton), 4 expressions</t>
+          <t>6 portraits du maire au choix (joueur_01 à 06), neutre seulement</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
+          <t>game/ui/portraits/joueur_*/</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>PNG 256×256</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
           <t>à confirmer</t>
         </is>
       </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>webp</t>
-        </is>
-      </c>
-      <c r="F5" s="2" t="inlineStr">
-        <is>
-          <t>Higgsfield</t>
-        </is>
-      </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Abonnement Higgsfield</t>
+          <t>à confirmer</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>Intégré</t>
+          <t>Provisoire</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>Session Godot</t>
-        </is>
-      </c>
-      <c r="J5" s="2" t="inlineStr"/>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>Cloud (brief) / Godot</t>
+        </is>
+      </c>
       <c r="K5" s="2" t="inlineStr">
         <is>
-          <t>Hebdo rural bienveillant (mordant 3)</t>
-        </is>
-      </c>
+          <t>Expressions à ajouter</t>
+        </is>
+      </c>
+      <c r="L5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -738,46 +755,47 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Décor</t>
+          <t>Portrait</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Studio TV</t>
+          <t>24 visages candidat_f01 à h12 (les 22 conseillers simples)</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>game/ui/decors/studio_tv.webp</t>
+          <t>game/ui/portraits/candidat_*/</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>webp</t>
+          <t>PNG 256×256</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>à confirmer</t>
+          <t>Higgsfield</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>à confirmer</t>
+          <t>Higgsfield</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>Intégré</t>
-        </is>
-      </c>
-      <c r="I6" s="2" t="inlineStr">
-        <is>
-          <t>Session Godot</t>
-        </is>
-      </c>
-      <c r="J6" s="2" t="inlineStr"/>
-      <c r="K6" s="2" t="n"/>
+          <t>Final</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr"/>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>Godot</t>
+        </is>
+      </c>
+      <c r="K6" s="2" t="inlineStr"/>
+      <c r="L6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -792,45 +810,42 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Studio radio</t>
+          <t>22 fonds (bureau du maire, mairie, panneaux, préfecture, conseil général, institutions, plateau JT, soirée électorale)</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>game/ui/decors/studio_radio.webp</t>
+          <t>game/ui/decors/</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>webp</t>
+          <t>WebP 1344×752</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>à confirmer</t>
+          <t>Higgsfield</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>à confirmer</t>
+          <t>Higgsfield</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>Intégré</t>
-        </is>
-      </c>
-      <c r="I7" s="2" t="inlineStr">
-        <is>
-          <t>Session Godot</t>
-        </is>
-      </c>
+          <t>Final</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr"/>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>Chemin déduit</t>
-        </is>
-      </c>
-      <c r="K7" s="2" t="n"/>
+          <t>Godot</t>
+        </is>
+      </c>
+      <c r="K7" s="2" t="inlineStr"/>
+      <c r="L7" s="2" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -845,45 +860,42 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Salle de meeting</t>
+          <t>studio_tv, studio_radio, meeting</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>game/ui/decors/meeting.webp</t>
+          <t>game/ui/decors/</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>webp</t>
+          <t>WebP 1600×900</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>à confirmer</t>
+          <t>Higgsfield</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>à confirmer</t>
+          <t>Higgsfield</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>Intégré</t>
-        </is>
-      </c>
-      <c r="I8" s="2" t="inlineStr">
-        <is>
-          <t>Session Godot</t>
-        </is>
-      </c>
+          <t>Final</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr"/>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>Chemin déduit</t>
-        </is>
-      </c>
-      <c r="K8" s="2" t="n"/>
+          <t>Godot</t>
+        </is>
+      </c>
+      <c r="K8" s="2" t="inlineStr"/>
+      <c r="L8" s="2" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -893,518 +905,520 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>UI</t>
+          <t>Décor</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Poste de télévision (presse)</t>
+          <t>Salle du conseil municipal</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>ui/presse/poste_tv.png</t>
+          <t>game/ui/decors/salle_conseil_municipal.webp</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>png</t>
+          <t>WebP</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>à confirmer</t>
+          <t>Fournie par Yannick</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>à confirmer</t>
+          <t>Projet</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>Intégré</t>
-        </is>
-      </c>
-      <c r="I9" s="2" t="inlineStr">
-        <is>
-          <t>Session Godot</t>
-        </is>
-      </c>
-      <c r="J9" s="2" t="inlineStr"/>
-      <c r="K9" s="2" t="n"/>
+          <t>Final</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr"/>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>Godot</t>
+        </is>
+      </c>
+      <c r="K9" s="2" t="inlineStr"/>
+      <c r="L9" s="2" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>TXT-001</t>
+          <t>IMG-009</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Texte</t>
+          <t>Décor</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Campagne : questions, réponses, journalistes</t>
+          <t>Hémicycle</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>game/data/campagne.json</t>
+          <t>game/ui/conseil/salle_hemicycle.webp</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>json</t>
+          <t>WebP 1920×1086</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Session Godot</t>
+          <t>Higgsfield</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>Projet</t>
+          <t>Higgsfield</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>Intégré</t>
-        </is>
-      </c>
-      <c r="I10" s="2" t="inlineStr">
-        <is>
-          <t>Session cloud (relecture)</t>
-        </is>
-      </c>
-      <c r="J10" s="2" t="inlineStr"/>
-      <c r="K10" s="2" t="n"/>
+          <t>Final</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr"/>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>Godot</t>
+        </is>
+      </c>
+      <c r="K10" s="2" t="inlineStr"/>
+      <c r="L10" s="2" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>TXT-002</t>
+          <t>IMG-010</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Texte</t>
+          <t>Illustration</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Presse et opinion</t>
+          <t>7 images d'événements</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>game/data/textes_opinion.json</t>
+          <t>game/ui/evenements/</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>json</t>
+          <t>WebP 1344×752</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Session Godot</t>
+          <t>Higgsfield</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>Projet</t>
+          <t>Higgsfield</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>Intégré</t>
-        </is>
-      </c>
-      <c r="I11" s="2" t="inlineStr">
-        <is>
-          <t>Session cloud (relecture)</t>
-        </is>
-      </c>
-      <c r="J11" s="2" t="inlineStr"/>
-      <c r="K11" s="2" t="n"/>
+          <t>Final</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr"/>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>Godot</t>
+        </is>
+      </c>
+      <c r="K11" s="2" t="inlineStr">
+        <is>
+          <t>À compléter si de nouveaux événements sont écrits</t>
+        </is>
+      </c>
+      <c r="L11" s="2" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>TXT-003</t>
+          <t>IMG-011</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Texte</t>
+          <t>Illustration</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Doléances des quartiers</t>
+          <t>5 unes du journal</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>game/data/doleances.json</t>
+          <t>game/ui/presse/</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>json</t>
+          <t>WebP 1168×880</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Session Godot</t>
+          <t>Higgsfield</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>Projet</t>
+          <t>Higgsfield</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>Intégré</t>
-        </is>
-      </c>
-      <c r="I12" s="2" t="inlineStr">
-        <is>
-          <t>Session cloud (relecture)</t>
-        </is>
-      </c>
-      <c r="J12" s="2" t="inlineStr"/>
-      <c r="K12" s="2" t="n"/>
+          <t>Final</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr"/>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>Godot</t>
+        </is>
+      </c>
+      <c r="K12" s="2" t="inlineStr"/>
+      <c r="L12" s="2" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>TXT-004</t>
+          <t>IMG-012</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Texte</t>
+          <t>UI</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Tutoriel</t>
+          <t>Poste de télévision de 1980, écran découpé</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>game/data/tutoriel.json</t>
+          <t>game/ui/presse/poste_tv.png</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>json</t>
+          <t>PNG</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Session Godot</t>
+          <t>Higgsfield</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>Projet</t>
+          <t>Higgsfield</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>Intégré</t>
-        </is>
-      </c>
-      <c r="I13" s="2" t="inlineStr">
-        <is>
-          <t>Session cloud (relecture)</t>
-        </is>
-      </c>
-      <c r="J13" s="2" t="inlineStr"/>
-      <c r="K13" s="2" t="n"/>
+          <t>Final</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr"/>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>Godot</t>
+        </is>
+      </c>
+      <c r="K13" s="2" t="inlineStr"/>
+      <c r="L13" s="2" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>TXT-005</t>
+          <t>IMG-013</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Texte</t>
+          <t>Carte</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Aides / infobulles</t>
+          <t>Carte de la commune (quartiers en polygones dans data/commune.json) et carte de France</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>game/data/aides.json</t>
+          <t>game/ui/.../carte_commune.webp, carte_france.webp</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>json</t>
+          <t>WebP 1024×688</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Session Godot</t>
+          <t>Higgsfield</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>Projet</t>
+          <t>Higgsfield</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>Intégré</t>
-        </is>
-      </c>
-      <c r="I14" s="2" t="inlineStr">
-        <is>
-          <t>Session cloud (relecture)</t>
-        </is>
-      </c>
-      <c r="J14" s="2" t="inlineStr"/>
-      <c r="K14" s="2" t="n"/>
+          <t>Final</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr"/>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>Godot</t>
+        </is>
+      </c>
+      <c r="K14" s="2" t="inlineStr"/>
+      <c r="L14" s="2" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>SND-001</t>
+          <t>IMG-014</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Son</t>
+          <t>Icônes</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Index des sons</t>
+          <t>16 icônes 128×128 et 16 médaillons 160×160</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>game/data/sons.json</t>
+          <t>à confirmer</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>json</t>
+          <t>PNG</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>Session Godot</t>
+          <t>Higgsfield</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>Projet</t>
+          <t>Higgsfield</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>Intégré</t>
-        </is>
-      </c>
-      <c r="I15" s="2" t="inlineStr">
-        <is>
-          <t>Session Godot</t>
-        </is>
-      </c>
-      <c r="J15" s="2" t="inlineStr"/>
-      <c r="K15" s="2" t="n"/>
+          <t>Final</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr"/>
+      <c r="J15" s="2" t="inlineStr">
+        <is>
+          <t>Godot</t>
+        </is>
+      </c>
+      <c r="K15" s="2" t="inlineStr"/>
+      <c r="L15" s="2" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>SND-010</t>
+          <t>IMG-015</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Son</t>
+          <t>Logo</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Applaudissements de meeting</t>
+          <t>Logo venatior_X studio</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>à définir</t>
+          <t>studio_logo.png</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>ogg</t>
+          <t>PNG</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>Recherche cloud</t>
+          <t>Fourni par Yannick</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>CC0 visé</t>
+          <t>Projet</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>Candidat trouvé</t>
-        </is>
-      </c>
-      <c r="I16" s="2" t="inlineStr">
-        <is>
-          <t>Session cloud</t>
-        </is>
-      </c>
+          <t>Final</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr"/>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>Voir onglet Sons à sourcer</t>
-        </is>
-      </c>
-      <c r="K16" s="2" t="inlineStr">
-        <is>
-          <t>La salle vous suit</t>
-        </is>
-      </c>
+          <t>Godot</t>
+        </is>
+      </c>
+      <c r="K16" s="2" t="inlineStr"/>
+      <c r="L16" s="2" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>SND-011</t>
+          <t>IMG-016</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Son</t>
+          <t>Logo</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Huées de meeting</t>
+          <t>Logo Godot (Andrea Calabró)</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>à définir</t>
+          <t>godot_logo.png</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>ogg</t>
+          <t>PNG</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>Recherche cloud</t>
+          <t>Godot</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>CC0 visé</t>
+          <t>CC BY 4.0, crédité</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>Recherche</t>
-        </is>
-      </c>
-      <c r="I17" s="2" t="inlineStr">
-        <is>
-          <t>Session cloud</t>
-        </is>
-      </c>
+          <t>Final</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr"/>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>Pas encore de CC0 sûr</t>
-        </is>
-      </c>
-      <c r="K17" s="2" t="inlineStr">
-        <is>
-          <t>La salle vous rejette</t>
-        </is>
-      </c>
+          <t>Godot</t>
+        </is>
+      </c>
+      <c r="K17" s="2" t="inlineStr"/>
+      <c r="L17" s="2" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>SND-012</t>
+          <t>IMG-017</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Son</t>
+          <t>Icône</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Jingles/ambiance par journaliste (presse, radio, TV)</t>
+          <t>Icône de l'exe</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>à définir</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>ogg</t>
+          <t>ico</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>Recherche cloud</t>
+          <t>Défaut Godot</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>CC0 visé</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>Recherche</t>
+          <t>Provisoire</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>Session cloud</t>
-        </is>
-      </c>
-      <c r="J18" s="2" t="inlineStr"/>
-      <c r="K18" s="2" t="n"/>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>Cloud</t>
+        </is>
+      </c>
+      <c r="K18" s="2" t="inlineStr"/>
+      <c r="L18" s="2" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>IMG-020</t>
+          <t>IMG-018</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Décor</t>
+          <t>Visuel de retour</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Place de la mairie, 4 états d'opinion (fête, normal, tendu, grève)</t>
+          <t>Tampons « Inscrite », « Adoptée », « Rejetée » ; lettre qui jaunit</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
@@ -1414,17 +1428,17 @@
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>webp</t>
+          <t>PNG</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>Higgsfield</t>
+          <t>à créer</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>Abonnement Higgsfield</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
@@ -1434,34 +1448,39 @@
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>Session cloud (brief) + Godot (intégration)</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="J19" s="2" t="inlineStr">
         <is>
-          <t>Narrative design, voir Lecons § 10.3</t>
+          <t>Cloud</t>
         </is>
       </c>
       <c r="K19" s="2" t="inlineStr">
         <is>
-          <t>L'opinion de la commune se voit sans chiffre</t>
+          <t>Voir onglet Signes et feedback</t>
+        </is>
+      </c>
+      <c r="L19" s="2" t="inlineStr">
+        <is>
+          <t>Le résultat d'un vote se voit</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>IMG-021</t>
+          <t>FNT-001</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Décor</t>
+          <t>Police</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Bureau du maire qui se remplit au fil du mandat (dossiers, coupures encadrées, lettres en souffrance)</t>
+          <t>Serif pour les titres (remplace Palatino Linotype système)</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
@@ -1471,17 +1490,17 @@
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>webp</t>
+          <t>TTF/OTF</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>Higgsfield</t>
+          <t>à choisir</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>Abonnement Higgsfield</t>
+          <t>SIL OFL visée</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
@@ -1491,34 +1510,35 @@
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>Session cloud (brief)</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr">
         <is>
-          <t>§ 10.3</t>
+          <t>Cloud</t>
         </is>
       </c>
       <c r="K20" s="2" t="inlineStr">
         <is>
-          <t>Le bilan du mandat se voit</t>
-        </is>
-      </c>
+          <t>Le rendu change d'un PC à l'autre tant qu'aucune police n'est embarquée</t>
+        </is>
+      </c>
+      <c r="L20" s="2" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>IMG-022</t>
+          <t>FNT-002</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Icônes</t>
+          <t>Police</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>Icônes des ressources et des modes de carte, style CK3</t>
+          <t>Sans-serif pour l'interface (remplace Segoe UI et la police Godot)</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
@@ -1528,17 +1548,17 @@
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>png/svg</t>
+          <t>TTF/OTF</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>à définir</t>
+          <t>à choisir</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>à définir</t>
+          <t>SIL OFL visée</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
@@ -1548,39 +1568,36 @@
       </c>
       <c r="I21" s="2" t="inlineStr">
         <is>
-          <t>Session cloud (recherche)</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="J21" s="2" t="inlineStr">
         <is>
-          <t>§ 10.5</t>
-        </is>
-      </c>
-      <c r="K21" s="2" t="inlineStr">
-        <is>
-          <t>Lire une ressource d'un coup d'œil</t>
-        </is>
-      </c>
+          <t>Cloud</t>
+        </is>
+      </c>
+      <c r="K21" s="2" t="inlineStr"/>
+      <c r="L21" s="2" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>MUS-001</t>
+          <t>SND-000</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Musique</t>
+          <t>Son</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Thèmes mairie et campagne avec cuivres de fanfare municipale en signature</t>
+          <t>64 sons décrits dans data/sons.json (9 musiques, 4 ambiances, 13 interface, 38 effets), déjà branchés : un .ogg au bon chemin joue aussitôt</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>à confirmer</t>
+          <t>game/.../musique|ambiance|interface|effets/</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
@@ -1590,64 +1607,65 @@
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>à définir</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>à définir</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>Recherche</t>
+          <t>Manquant</t>
         </is>
       </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
-          <t>Session cloud</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="J22" s="2" t="inlineStr">
         <is>
-          <t>Brief § 10.5 ; vérifier ce qui existe déjà</t>
+          <t>Cloud</t>
         </is>
       </c>
       <c r="K22" s="2" t="inlineStr">
         <is>
-          <t>L'ambiance du mandat (fête ou grève)</t>
-        </is>
-      </c>
+          <t>Le jeu est muet. Détail des 17 prioritaires dans l'onglet Sons à sourcer</t>
+        </is>
+      </c>
+      <c r="L22" s="2" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>DOC-001</t>
+          <t>TXT-001</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>Document</t>
+          <t>Texte</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Bible graphique de Politics</t>
+          <t>campagne.json : 18 types de questions × 2 textes + relance ; attaques, résumés, répliques, réactions, discours</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>politics-assets/</t>
+          <t>game/data/campagne.json</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>md</t>
+          <t>json</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>Session cloud + Godot</t>
+          <t>Claude (Godot)</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
@@ -1657,50 +1675,55 @@
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>Manquant</t>
+          <t>À relire</t>
         </is>
       </c>
       <c r="I23" s="2" t="inlineStr">
         <is>
-          <t>Session cloud (brouillon)</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="J23" s="2" t="inlineStr">
         <is>
-          <t>Besoin de captures du jeu</t>
-        </is>
-      </c>
-      <c r="K23" s="2" t="inlineStr"/>
+          <t>Cloud</t>
+        </is>
+      </c>
+      <c r="K23" s="2" t="inlineStr">
+        <is>
+          <t>Variantes à écrire</t>
+        </is>
+      </c>
+      <c r="L23" s="2" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>DOC-002</t>
+          <t>TXT-002</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>Document</t>
+          <t>Texte</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Game pillars de Politics</t>
+          <t>textes_opinion.json : 32 lettres d'habitants, 39 gabarits de presse</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>Lecons_videos_game_design.md § 10.1</t>
+          <t>game/data/textes_opinion.json</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>md</t>
+          <t>json</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>Session cloud</t>
+          <t>Claude (Godot)</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
@@ -1710,46 +1733,51 @@
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>Provisoire</t>
+          <t>À relire</t>
         </is>
       </c>
       <c r="I24" s="2" t="inlineStr">
         <is>
-          <t>Yannick (validation)</t>
-        </is>
-      </c>
-      <c r="J24" s="2" t="inlineStr"/>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="J24" s="2" t="inlineStr">
+        <is>
+          <t>Cloud</t>
+        </is>
+      </c>
       <c r="K24" s="2" t="inlineStr"/>
+      <c r="L24" s="2" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>DOC-003</t>
+          <t>TXT-003</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>Document</t>
+          <t>Texte</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>Pitch du jeu (long et court)</t>
+          <t>doleances.json : 5 porte-parole, 7 lettres</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>Lecons_videos_game_design.md § 11.3</t>
+          <t>game/data/doleances.json</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>md</t>
+          <t>json</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>Session cloud</t>
+          <t>Claude (Godot)</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
@@ -1759,50 +1787,51 @@
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>Provisoire</t>
+          <t>À relire</t>
         </is>
       </c>
       <c r="I25" s="2" t="inlineStr">
         <is>
-          <t>Yannick (validation)</t>
-        </is>
-      </c>
-      <c r="J25" s="2" t="inlineStr"/>
-      <c r="K25" s="2" t="inlineStr">
-        <is>
-          <t>Donner envie en une minute</t>
-        </is>
-      </c>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="J25" s="2" t="inlineStr">
+        <is>
+          <t>Cloud</t>
+        </is>
+      </c>
+      <c r="K25" s="2" t="inlineStr"/>
+      <c r="L25" s="2" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>DOC-004</t>
+          <t>TXT-004</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>Document</t>
+          <t>Texte</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Protocole et questionnaire de playtest</t>
+          <t>evenements.json : seulement 6 événements pour 3 ans de jeu</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>à rédiger</t>
+          <t>game/data/evenements.json</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>md</t>
+          <t>json</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>Session cloud</t>
+          <t>Claude (Godot)</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
@@ -1812,85 +1841,696 @@
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>Manquant</t>
+          <t>Insuffisant</t>
         </is>
       </c>
       <c r="I26" s="2" t="inlineStr">
         <is>
-          <t>Session cloud</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="J26" s="2" t="inlineStr">
         <is>
-          <t>§ 11.8</t>
-        </is>
-      </c>
-      <c r="K26" s="2" t="inlineStr"/>
+          <t>Cloud</t>
+        </is>
+      </c>
+      <c r="K26" s="2" t="inlineStr">
+        <is>
+          <t>Écrire les événements historiques 1980-1983 et les crises locales</t>
+        </is>
+      </c>
+      <c r="L26" s="2" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
+          <t>TXT-005</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>Texte</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>aides.json : 14 explications</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>game/data/aides.json</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>json</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>Claude (Godot)</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t>Projet</t>
+        </is>
+      </c>
+      <c r="H27" s="2" t="inlineStr">
+        <is>
+          <t>À relire</t>
+        </is>
+      </c>
+      <c r="I27" s="2" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="J27" s="2" t="inlineStr">
+        <is>
+          <t>Cloud</t>
+        </is>
+      </c>
+      <c r="K27" s="2" t="inlineStr">
+        <is>
+          <t>Version courte, 2-3 phrases</t>
+        </is>
+      </c>
+      <c r="L27" s="2" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>TXT-006</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>Texte</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>tutoriel.json : 26 étapes de visite, 11 premiers pas</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>game/data/tutoriel.json</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>json</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>Claude (Godot)</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>Projet</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="inlineStr">
+        <is>
+          <t>À relire</t>
+        </is>
+      </c>
+      <c r="I28" s="2" t="inlineStr"/>
+      <c r="J28" s="2" t="inlineStr">
+        <is>
+          <t>Cloud</t>
+        </is>
+      </c>
+      <c r="K28" s="2" t="inlineStr"/>
+      <c r="L28" s="2" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>TXT-007</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>Texte</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>carnet.json (21 chapitres), dialogues.json (28 situations), textes_ui.json (362 libellés)</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>game/data/</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>json</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>Claude (Godot)</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t>Projet</t>
+        </is>
+      </c>
+      <c r="H29" s="2" t="inlineStr">
+        <is>
+          <t>À relire</t>
+        </is>
+      </c>
+      <c r="I29" s="2" t="inlineStr"/>
+      <c r="J29" s="2" t="inlineStr">
+        <is>
+          <t>Cloud</t>
+        </is>
+      </c>
+      <c r="K29" s="2" t="inlineStr"/>
+      <c r="L29" s="2" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>IMG-020</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>Décor</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>Place de la mairie, 4 états d'opinion (fête, normal, tendu, grève)</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>à définir</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>webp</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>Higgsfield</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t>Abonnement Higgsfield</t>
+        </is>
+      </c>
+      <c r="H30" s="2" t="inlineStr">
+        <is>
+          <t>Manquant</t>
+        </is>
+      </c>
+      <c r="I30" s="2" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="J30" s="2" t="inlineStr">
+        <is>
+          <t>Session cloud (brief) + Godot (intégration)</t>
+        </is>
+      </c>
+      <c r="K30" s="2" t="inlineStr">
+        <is>
+          <t>Narrative design, voir Lecons § 10.3</t>
+        </is>
+      </c>
+      <c r="L30" s="2" t="inlineStr">
+        <is>
+          <t>L'opinion de la commune se voit sans chiffre</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>IMG-021</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>Décor</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>Bureau du maire qui se remplit au fil du mandat (dossiers, coupures encadrées, lettres en souffrance)</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>à définir</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>webp</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>Higgsfield</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="inlineStr">
+        <is>
+          <t>Abonnement Higgsfield</t>
+        </is>
+      </c>
+      <c r="H31" s="2" t="inlineStr">
+        <is>
+          <t>Manquant</t>
+        </is>
+      </c>
+      <c r="I31" s="2" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="J31" s="2" t="inlineStr">
+        <is>
+          <t>Session cloud (brief)</t>
+        </is>
+      </c>
+      <c r="K31" s="2" t="inlineStr">
+        <is>
+          <t>§ 10.3</t>
+        </is>
+      </c>
+      <c r="L31" s="2" t="inlineStr">
+        <is>
+          <t>Le bilan du mandat se voit</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>IMG-022</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>Icônes</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>Icônes des ressources et des modes de carte, style CK3</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>à définir</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>png/svg</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>à définir</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t>à définir</t>
+        </is>
+      </c>
+      <c r="H32" s="2" t="inlineStr">
+        <is>
+          <t>Manquant</t>
+        </is>
+      </c>
+      <c r="I32" s="2" t="inlineStr"/>
+      <c r="J32" s="2" t="inlineStr">
+        <is>
+          <t>Session cloud (recherche)</t>
+        </is>
+      </c>
+      <c r="K32" s="2" t="inlineStr">
+        <is>
+          <t>§ 10.5</t>
+        </is>
+      </c>
+      <c r="L32" s="2" t="inlineStr">
+        <is>
+          <t>Lire une ressource d'un coup d'œil</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>MUS-001</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>Musique</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>Thèmes mairie et campagne avec cuivres de fanfare municipale en signature</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>à confirmer</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>ogg</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>à définir</t>
+        </is>
+      </c>
+      <c r="G33" s="2" t="inlineStr">
+        <is>
+          <t>à définir</t>
+        </is>
+      </c>
+      <c r="H33" s="2" t="inlineStr">
+        <is>
+          <t>Recherche</t>
+        </is>
+      </c>
+      <c r="I33" s="2" t="inlineStr"/>
+      <c r="J33" s="2" t="inlineStr">
+        <is>
+          <t>Session cloud</t>
+        </is>
+      </c>
+      <c r="K33" s="2" t="inlineStr">
+        <is>
+          <t>Brief § 10.5 ; vérifier ce qui existe déjà</t>
+        </is>
+      </c>
+      <c r="L33" s="2" t="inlineStr">
+        <is>
+          <t>L'ambiance du mandat (fête ou grève)</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>DOC-001</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>Document</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>Bible graphique de Politics</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>politics-assets/</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>md</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>Session cloud + Godot</t>
+        </is>
+      </c>
+      <c r="G34" s="2" t="inlineStr">
+        <is>
+          <t>Projet</t>
+        </is>
+      </c>
+      <c r="H34" s="2" t="inlineStr">
+        <is>
+          <t>Manquant</t>
+        </is>
+      </c>
+      <c r="I34" s="2" t="inlineStr"/>
+      <c r="J34" s="2" t="inlineStr">
+        <is>
+          <t>Session cloud (brouillon)</t>
+        </is>
+      </c>
+      <c r="K34" s="2" t="inlineStr">
+        <is>
+          <t>Besoin de captures du jeu</t>
+        </is>
+      </c>
+      <c r="L34" s="2" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>DOC-002</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>Document</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>Game pillars de Politics</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>Lecons_videos_game_design.md § 10.1</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>md</t>
+        </is>
+      </c>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t>Session cloud</t>
+        </is>
+      </c>
+      <c r="G35" s="2" t="inlineStr">
+        <is>
+          <t>Projet</t>
+        </is>
+      </c>
+      <c r="H35" s="2" t="inlineStr">
+        <is>
+          <t>Provisoire</t>
+        </is>
+      </c>
+      <c r="I35" s="2" t="inlineStr"/>
+      <c r="J35" s="2" t="inlineStr">
+        <is>
+          <t>Yannick (validation)</t>
+        </is>
+      </c>
+      <c r="K35" s="2" t="n"/>
+      <c r="L35" s="2" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>DOC-003</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>Document</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>Pitch du jeu (long et court)</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>Lecons_videos_game_design.md § 11.3</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>md</t>
+        </is>
+      </c>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>Session cloud</t>
+        </is>
+      </c>
+      <c r="G36" s="2" t="inlineStr">
+        <is>
+          <t>Projet</t>
+        </is>
+      </c>
+      <c r="H36" s="2" t="inlineStr">
+        <is>
+          <t>Provisoire</t>
+        </is>
+      </c>
+      <c r="I36" s="2" t="inlineStr"/>
+      <c r="J36" s="2" t="inlineStr">
+        <is>
+          <t>Yannick (validation)</t>
+        </is>
+      </c>
+      <c r="K36" s="2" t="n"/>
+      <c r="L36" s="2" t="inlineStr">
+        <is>
+          <t>Donner envie en une minute</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>DOC-004</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>Document</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>Protocole et questionnaire de playtest</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>à rédiger</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>md</t>
+        </is>
+      </c>
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t>Session cloud</t>
+        </is>
+      </c>
+      <c r="G37" s="2" t="inlineStr">
+        <is>
+          <t>Projet</t>
+        </is>
+      </c>
+      <c r="H37" s="2" t="inlineStr">
+        <is>
+          <t>Manquant</t>
+        </is>
+      </c>
+      <c r="I37" s="2" t="inlineStr"/>
+      <c r="J37" s="2" t="inlineStr">
+        <is>
+          <t>Session cloud</t>
+        </is>
+      </c>
+      <c r="K37" s="2" t="inlineStr">
+        <is>
+          <t>§ 11.8</t>
+        </is>
+      </c>
+      <c r="L37" s="2" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
           <t>DOC-005</t>
         </is>
       </c>
-      <c r="B27" s="2" t="inlineStr">
+      <c r="B38" s="2" t="inlineStr">
         <is>
           <t>Maquettes</t>
         </is>
       </c>
-      <c r="C27" s="2" t="inlineStr">
+      <c r="C38" s="2" t="inlineStr">
         <is>
           <t>Maquettes d'écrans avant code (fiche de quartier, trois horizons, front électoral)</t>
         </is>
       </c>
-      <c r="D27" s="2" t="inlineStr">
+      <c r="D38" s="2" t="inlineStr">
         <is>
           <t>à faire</t>
         </is>
       </c>
-      <c r="E27" s="2" t="inlineStr">
+      <c r="E38" s="2" t="inlineStr">
         <is>
           <t>png</t>
         </is>
       </c>
-      <c r="F27" s="2" t="inlineStr">
+      <c r="F38" s="2" t="inlineStr">
         <is>
           <t>Session cloud</t>
         </is>
       </c>
-      <c r="G27" s="2" t="inlineStr">
+      <c r="G38" s="2" t="inlineStr">
         <is>
           <t>Projet</t>
         </is>
       </c>
-      <c r="H27" s="2" t="inlineStr">
+      <c r="H38" s="2" t="inlineStr">
         <is>
           <t>Manquant</t>
         </is>
       </c>
-      <c r="I27" s="2" t="inlineStr">
+      <c r="I38" s="2" t="inlineStr"/>
+      <c r="J38" s="2" t="inlineStr">
         <is>
           <t>Session cloud</t>
         </is>
       </c>
-      <c r="J27" s="2" t="inlineStr">
+      <c r="K38" s="2" t="inlineStr">
         <is>
           <t>§ 11.4, à valider par Yannick avant code</t>
         </is>
       </c>
-      <c r="K27" s="2" t="inlineStr">
+      <c r="L38" s="2" t="inlineStr">
         <is>
           <t>Juger une idée avant de la coder</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K27"/>
-  <dataValidations count="1">
-    <dataValidation sqref="H2:H500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Manquant,Recherche,Candidat trouvé,Livré à la session Godot,Intégré,Final,Provisoire"</formula1>
-    </dataValidation>
-  </dataValidations>
+  <autoFilter ref="A1:L38"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1912,7 +2552,7 @@
     <col width="36" customWidth="1" min="6" max="6"/>
     <col width="34" customWidth="1" min="7" max="7"/>
     <col width="30" customWidth="1" min="8" max="8"/>
-    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="60" customWidth="1" min="9" max="9"/>
     <col width="16" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
@@ -2011,12 +2651,12 @@
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>à confirmer</t>
+          <t>En partie. Existe : coût U, délai, effets par quartier, raison du refus. Manque : élus concernés, animation, son papier</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>Manquant</t>
+          <t>À compléter</t>
         </is>
       </c>
     </row>
@@ -2063,12 +2703,12 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>à confirmer</t>
+          <t>En partie. Existe : message « Inscrite à la séance du … », date. Son effets/tampon au catalogue sans fichier. Manque : tampon animé</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>Manquant</t>
+          <t>À compléter</t>
         </is>
       </c>
     </row>
@@ -2115,7 +2755,7 @@
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>En partie</t>
+          <t>En partie. Existe : relation, disposition, confiance, alliance, 12 expressions en fondu, effets verts/gris. Manque : ambition, chiffre rouge, sons rencontre et porte_bureau</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
@@ -2167,12 +2807,12 @@
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>à confirmer</t>
+          <t>En partie. Existe : décompte prévu, vote siège par siège, résultat vert/rouge, sièges retournés cerclés avec portraits. Sons branchés sans fichier. Manque : tampon Adoptée/Rejetée, secousse</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>Manquant</t>
+          <t>À compléter</t>
         </is>
       </c>
     </row>
@@ -2219,7 +2859,7 @@
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>En partie</t>
+          <t>En partie. Existe : compétence, écart, bonus/malus. Manque : écharpe, carillon (pas au catalogue)</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
@@ -2271,12 +2911,12 @@
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>à confirmer</t>
+          <t>En partie. Existe : lettre, date limite, « Doléance sans réponse » au journal, tension. Son courrier sans fichier. Manque : lettre qui jaunit, cachet</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>Manquant</t>
+          <t>À compléter</t>
         </is>
       </c>
     </row>
@@ -2323,12 +2963,12 @@
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>à confirmer</t>
+          <t>En partie. Existe : modes de carte (popularité, satisfaction, besoin, tension, contrôle), tension sur hausse d'impôts. Manque : infobulle d'effet prévu, animation, calculatrice</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>Manquant</t>
+          <t>À compléter</t>
         </is>
       </c>
     </row>
@@ -2375,7 +3015,7 @@
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>En partie (journal)</t>
+          <t>En partie. Pas de bouton : temps continu (pause, ×1 à ×3, 1 mois = 1 min). Existe : une du journal, JT national, notifications 8 s. Son rotative sans fichier. Manque : journal qui tombe</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
@@ -2427,12 +3067,12 @@
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>Non</t>
+          <t>En partie. Existe : événement « Dissidence dans la majorité » (confiance de Mérieux &lt; 25), journal, portrait teinté par groupe. Manque : bruits de couloir génériques, porte qui claque</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>Manquant</t>
+          <t>À compléter</t>
         </is>
       </c>
     </row>
@@ -2479,7 +3119,7 @@
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>En partie</t>
+          <t>En partie. Existe : tension par quartier, cortège sur carte tactique tour par tour, issues. Sons cortege, affrontement, negociation, ambiance/manifestation sans fichier</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
@@ -2531,7 +3171,7 @@
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>En partie</t>
+          <t>En partie. Existe : chance, gain, risque, 4 expressions, relance, hochement, score coloré, jauge. Sons interview, debat sans fichier. Manque : stylo, jingle radio, générique TV</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
@@ -2583,12 +3223,12 @@
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>En partie</t>
+          <t>En partie. Existe : 3 soucis du quartier, décor, interpellation, jauge. Manque : applaudissements, huées, chaises</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>Candidat trouvé</t>
+          <t>À compléter</t>
         </is>
       </c>
     </row>
@@ -2635,7 +3275,7 @@
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>En partie</t>
+          <t>En partie. Existe : expressions de Carminati, attaque sur le pire du bilan. Son debat sans fichier. Manque : annonce du fait à l'avance, cadrages, générique</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
@@ -2687,12 +3327,12 @@
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>à confirmer</t>
+          <t>En partie. Existe : coût (sondage 0,2 U, tract gratuit), sondages en texte. Son tract sans fichier. Manque : courbe animée</t>
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>Manquant</t>
+          <t>À compléter</t>
         </is>
       </c>
     </row>
@@ -2739,12 +3379,12 @@
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>à confirmer</t>
+          <t>En partie. Existe : résultats des deux tours, JT « Le verdict des urnes », une, Bilan du mandat. Musiques victoire/défaite sans fichier. Manque : compte à rebours, résultats par quartier, une Réélu/Battu</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>Manquant</t>
+          <t>À compléter</t>
         </is>
       </c>
     </row>
@@ -2760,6 +3400,900 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G35"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="44" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="9" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>Chemin (sous le dossier sons)</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>Priorité</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>Statut</t>
+        </is>
+      </c>
+      <c r="E1" s="4" t="inlineStr">
+        <is>
+          <t>Candidat / source</t>
+        </is>
+      </c>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
+          <t>Licence</t>
+        </is>
+      </c>
+      <c r="G1" s="4" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>musique/menu.ogg</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>musique</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Manquant</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>musique/intro.ogg</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>musique</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Manquant</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>musique/mairie.ogg</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>musique</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Manquant</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>interface/clic.ogg</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>interface</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Manquant</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>interface/panneau_ouvrir.ogg</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>interface</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Manquant</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>interface/panneau_fermer.ogg</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>interface</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Manquant</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>interface/notification.ogg</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>interface</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Manquant</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>effets/conseil_cloche.ogg</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>effets</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Manquant</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>effets/vote_marteau.ogg</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>effets</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Manquant</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>effets/vote_adoptee.ogg</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>effets</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Manquant</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>effets/vote_rejetee.ogg</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>effets</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Manquant</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>effets/inauguration.ogg</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>effets</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Manquant</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>effets/evenement.ogg</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>effets</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Manquant</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>effets/cortege.ogg</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>effets</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Manquant</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>effets/journal.ogg</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>effets</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Manquant</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>effets/jt_generique.ogg</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>effets</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Manquant</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>effets/election_resultat.ogg</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>effets</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Manquant</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>effets/applaudissements_meeting.ogg (à ajouter au catalogue)</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>effets</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Manquant</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Pas encore dans sons.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>effets/huees_meeting.ogg (à ajouter au catalogue)</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>effets</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Manquant</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>Pas encore dans sons.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>effets/stylo_carnet.ogg (à ajouter au catalogue)</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>effets</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Manquant</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>Pas encore dans sons.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>effets/jingle_radio_libre.ogg (à ajouter au catalogue)</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>effets</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Manquant</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>Pas encore dans sons.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>effets/generique_debat.ogg (à ajouter au catalogue)</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>effets</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Manquant</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>Pas encore dans sons.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>effets/public_rires_murmures.ogg (à ajouter au catalogue)</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>effets</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Manquant</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>Pas encore dans sons.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>effets/tampon.ogg</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>effets</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Manquant</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>Déjà au catalogue</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>effets/rotative.ogg</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>effets</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Manquant</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>Déjà au catalogue</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>effets/porte_bureau.ogg</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>effets</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Manquant</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>Déjà au catalogue</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>effets/machine_a_ecrire.ogg</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>effets</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Manquant</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>Déjà au catalogue</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>effets/interview.ogg</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>effets</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Manquant</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>Déjà au catalogue</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>effets/debat.ogg</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>effets</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Manquant</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>Déjà au catalogue</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>effets/tract.ogg</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>effets</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Manquant</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>Déjà au catalogue</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>effets/sondage.ogg</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>effets</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Manquant</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>Déjà au catalogue</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>effets/courrier.ogg</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>effets</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Manquant</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>Déjà au catalogue</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>ambiance/conseil.ogg</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>ambiance</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Manquant</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>Déjà au catalogue</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>ambiance/manifestation.ogg</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>ambiance</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Manquant</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>Déjà au catalogue</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:G35"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3525,7 +5059,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3805,7 +5339,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
List CC0 music candidates for Politics in the asset tracker
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013ScbAjnnHvWadm23zH5KKB
</commit_message>
<xml_diff>
--- a/politics-assets/Politics_assets.xlsx
+++ b/politics-assets/Politics_assets.xlsx
@@ -11,16 +11,17 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Signes et feedback" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sons prioritaires" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sons à sourcer" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Textes à écrire" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide GSG" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Musiques à sourcer" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Textes à écrire" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide GSG" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventaire'!$A$1:$L$38</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Signes et feedback'!$A$1:$J$16</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Sons prioritaires'!$A$1:$G$35</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Sons à sourcer'!$A$1:$I$17</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Textes à écrire'!$A$1:$F$8</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Guide GSG'!$A$1:$E$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Textes à écrire'!$A$1:$F$8</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Guide GSG'!$A$1:$E$13</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -5065,6 +5066,235 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:E8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="50" customWidth="1" min="2" max="2"/>
+    <col width="52" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>Usage visé</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>Candidat</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>URL</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>Licence annoncée</t>
+        </is>
+      </c>
+      <c r="E1" s="4" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>musique/menu</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>« vintage menu », synthwave lo-fi, environ 5 min</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>https://opengameart.org/content/vintage-menu</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>CC0 (à vérifier sur la page)</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Pas besoin de boucle</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>musique/menu ou intro</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>« Of Far Different Nature - Oldskool », synthé rétro des années 80</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>https://opengameart.org/node/107451</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>CC0 (à vérifier)</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Un commentaire le recommande pour un menu ; nœud à confirmer</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>musique/menu</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>« menu music 1 », boucle batterie et synthés</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>https://opengameart.org/content/menu-music-1</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>CC0 / domaine public (à vérifier)</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>musique/campagne</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>« some militaristic tune », cuivres et tambours</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>https://opengameart.org/content/some-militaristic-tune</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>CC0 (à vérifier)</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>Plus martial que fanfare municipale</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>musique/campagne</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Marche lente en boucle, environ 4 min</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>https://opengameart.org/node/10683</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>CC0 (à vérifier)</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>musique/mairie</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>« jazz n brass loop »</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>https://opengameart.org/content/jazz-n-brass-loop</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>CC0 (à vérifier)</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>Plutôt jazzy années 90</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>musique/* (banque)</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>FreePD : banque de musiques CC0, avec un filtre CC0 dans sa recherche</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>https://freepd.com</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>CC0 annoncé ; conditions de téléchargement à vérifier</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>Catégories : comédie, sentimental, électronique, upbeat…</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:F8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -5339,7 +5569,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>